<commit_message>
Finsih run testing on series
</commit_message>
<xml_diff>
--- a/RunningTimeRecord.xlsx
+++ b/RunningTimeRecord.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\MONASH\Year_3_sem_1\FIT3143\Week 04\FIT3143_lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62499079-4B7C-42CF-B560-9A89B60CE0AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C4B2AED-CA77-417B-9CBF-A83EF2921DE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -147,13 +147,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -163,6 +157,12 @@
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -457,18 +457,18 @@
       <c r="C1" s="1"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4" t="s">
+      <c r="C3" s="12"/>
+      <c r="D3" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4" t="s">
+      <c r="E3" s="12"/>
+      <c r="F3" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="4"/>
+      <c r="G3" s="12"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
@@ -716,212 +716,248 @@
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
     </row>
-    <row r="16" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="5"/>
-      <c r="B16" s="6" t="s">
+    <row r="16" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="4"/>
+      <c r="B16" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6" t="s">
+      <c r="C16" s="13"/>
+      <c r="D16" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6" t="s">
+      <c r="E16" s="13"/>
+      <c r="F16" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="G16" s="6"/>
-    </row>
-    <row r="17" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="8" t="s">
+      <c r="G16" s="13"/>
+    </row>
+    <row r="17" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="G17" s="6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:7" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="11">
+    <row r="18" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="9">
         <v>10000000</v>
       </c>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12">
+      <c r="B18" s="10">
+        <v>3.778915</v>
+      </c>
+      <c r="C18" s="10">
+        <v>8.6425140000000003</v>
+      </c>
+      <c r="D18" s="10">
         <v>0.188636</v>
       </c>
-      <c r="E18" s="12">
+      <c r="E18" s="10">
         <v>4.9392230000000001</v>
       </c>
-      <c r="F18" s="12">
+      <c r="F18" s="10">
         <v>1.384317</v>
       </c>
-      <c r="G18" s="12">
+      <c r="G18" s="10">
         <v>6.1650879999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="10">
+    <row r="19" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="8">
         <v>15000000</v>
       </c>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5">
+      <c r="B19" s="4">
+        <v>6.2206219999999997</v>
+      </c>
+      <c r="C19" s="4">
+        <v>13.401472999999999</v>
+      </c>
+      <c r="D19" s="4">
         <v>0.30043999999999998</v>
       </c>
-      <c r="E19" s="5">
+      <c r="E19" s="4">
         <v>8.0359610000000004</v>
       </c>
-      <c r="F19" s="5">
+      <c r="F19" s="4">
         <v>2.5880679999999998</v>
       </c>
-      <c r="G19" s="5">
+      <c r="G19" s="4">
         <v>10.625273</v>
       </c>
     </row>
-    <row r="20" spans="1:7" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="11">
+    <row r="20" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="9">
         <v>20000000</v>
       </c>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12">
+      <c r="B20" s="10">
+        <v>10.102762</v>
+      </c>
+      <c r="C20" s="10">
+        <v>19.441248000000002</v>
+      </c>
+      <c r="D20" s="10">
         <v>0.446938</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="10">
         <v>10.283652</v>
       </c>
-      <c r="F20" s="12">
+      <c r="F20" s="10">
         <v>2.7769949999999999</v>
       </c>
-      <c r="G20" s="12">
+      <c r="G20" s="10">
         <v>12.613759999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="10">
+    <row r="21" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="8">
         <v>25000000</v>
       </c>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5">
+      <c r="B21" s="4">
+        <v>13.203678</v>
+      </c>
+      <c r="C21" s="4">
+        <v>25.747924000000001</v>
+      </c>
+      <c r="D21" s="4">
         <v>0.60850400000000004</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E21" s="4">
         <v>11.7872</v>
       </c>
-      <c r="F21" s="5">
+      <c r="F21" s="4">
         <v>3.9838559999999998</v>
       </c>
-      <c r="G21" s="5">
+      <c r="G21" s="4">
         <v>16.541592000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:7" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="11">
+    <row r="22" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="9">
         <v>30000000</v>
       </c>
-      <c r="B22" s="12"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12">
+      <c r="B22" s="10">
+        <v>17.911546000000001</v>
+      </c>
+      <c r="C22" s="10">
+        <v>30.626833000000001</v>
+      </c>
+      <c r="D22" s="10">
         <v>0.78666400000000003</v>
       </c>
-      <c r="E22" s="12">
+      <c r="E22" s="10">
         <v>16.037421999999999</v>
       </c>
-      <c r="F22" s="12">
+      <c r="F22" s="10">
         <v>5.5545479999999996</v>
       </c>
-      <c r="G22" s="12">
+      <c r="G22" s="10">
         <v>19.275448000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="10">
+    <row r="23" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="8">
         <v>35000000</v>
       </c>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5">
+      <c r="B23" s="4">
+        <v>19.685684999999999</v>
+      </c>
+      <c r="C23" s="4">
+        <v>35.967072999999999</v>
+      </c>
+      <c r="D23" s="4">
         <v>0.97917200000000004</v>
       </c>
-      <c r="E23" s="5">
+      <c r="E23" s="4">
         <v>16.859352000000001</v>
       </c>
-      <c r="F23" s="5">
+      <c r="F23" s="4">
         <v>6.1012940000000002</v>
       </c>
-      <c r="G23" s="5">
+      <c r="G23" s="4">
         <v>22.961316</v>
       </c>
     </row>
-    <row r="24" spans="1:7" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="11">
+    <row r="24" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="9">
         <v>40000000</v>
       </c>
-      <c r="B24" s="12"/>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12">
+      <c r="B24" s="10">
+        <v>26.964960999999999</v>
+      </c>
+      <c r="C24" s="10">
+        <v>47.716700000000003</v>
+      </c>
+      <c r="D24" s="10">
         <v>1.135345</v>
       </c>
-      <c r="E24" s="12">
+      <c r="E24" s="10">
         <v>22.491413999999999</v>
       </c>
-      <c r="F24" s="12">
+      <c r="F24" s="10">
         <v>6.5744150000000001</v>
       </c>
-      <c r="G24" s="12">
+      <c r="G24" s="10">
         <v>25.531298</v>
       </c>
     </row>
-    <row r="25" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="10">
+    <row r="25" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="8">
         <v>45000000</v>
       </c>
-      <c r="B25" s="5"/>
-      <c r="C25" s="5"/>
-      <c r="D25" s="5">
+      <c r="B25" s="4">
+        <v>31.982582000000001</v>
+      </c>
+      <c r="C25" s="4">
+        <v>55.762712000000001</v>
+      </c>
+      <c r="D25" s="4">
         <v>1.3597349999999999</v>
       </c>
-      <c r="E25" s="5">
+      <c r="E25" s="4">
         <v>24.880361000000001</v>
       </c>
-      <c r="F25" s="5">
+      <c r="F25" s="4">
         <v>7.7472500000000002</v>
       </c>
-      <c r="G25" s="5">
+      <c r="G25" s="4">
         <v>31.823687</v>
       </c>
     </row>
-    <row r="26" spans="1:7" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="11">
+    <row r="26" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="9">
         <v>50000000</v>
       </c>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12">
+      <c r="B26" s="10">
+        <v>33.868523000000003</v>
+      </c>
+      <c r="C26" s="10">
+        <v>57.504927000000002</v>
+      </c>
+      <c r="D26" s="10">
         <v>1.552114</v>
       </c>
-      <c r="E26" s="12">
+      <c r="E26" s="10">
         <v>25.495045000000001</v>
       </c>
-      <c r="F26" s="12">
+      <c r="F26" s="10">
         <v>9.0593489999999992</v>
       </c>
-      <c r="G26" s="12">
+      <c r="G26" s="10">
         <v>31.419589999999999</v>
       </c>
     </row>
@@ -954,14 +990,14 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4" t="s">
+      <c r="C3" s="12"/>
+      <c r="D3" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="4"/>
+      <c r="E3" s="12"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
@@ -1091,14 +1127,14 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4" t="s">
+      <c r="C14" s="12"/>
+      <c r="D14" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="E14" s="4"/>
+      <c r="E14" s="12"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">

</xml_diff>

<commit_message>
Implement auto testing file
</commit_message>
<xml_diff>
--- a/RunningTimeRecord.xlsx
+++ b/RunningTimeRecord.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chtay\Documents\FIT3143\FIT3143_lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EBB60A7-49C7-4CBF-98A7-5BD253E40718}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A6E0418-6ABA-4BA1-80CB-AD25423B853B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="10060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="13">
   <si>
     <t>n</t>
   </si>
@@ -91,7 +91,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -101,6 +101,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -117,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -130,10 +136,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -416,611 +426,902 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="8" width="22.6328125" customWidth="1"/>
+    <col min="1" max="6" width="22.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B3" s="7" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7" t="s">
+      <c r="C3" s="8"/>
+      <c r="D3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H3" s="6"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="6" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="6" t="s">
         <v>2</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>10000000</v>
       </c>
       <c r="B5">
-        <v>4.1623950000000001</v>
-      </c>
-      <c r="C5">
-        <f>5.247637+B5</f>
-        <v>9.4100320000000011</v>
-      </c>
+        <v>4.221819</v>
+      </c>
+      <c r="C5" s="7"/>
       <c r="D5">
-        <v>0.68708499999999995</v>
-      </c>
-      <c r="E5">
-        <v>4.681508</v>
-      </c>
+        <v>0.66401900000000003</v>
+      </c>
+      <c r="E5" s="7"/>
       <c r="F5">
         <f>B5/D5</f>
-        <v>6.058049586295728</v>
-      </c>
-      <c r="G5" s="5">
-        <v>1.446939</v>
-      </c>
-      <c r="H5" s="5">
-        <v>6.7915789999999996</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+        <v>6.3579792144501885</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
+        <v>11000000</v>
+      </c>
+      <c r="B6">
+        <v>4.7456699999999996</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6">
+        <v>0.76085100000000006</v>
+      </c>
+      <c r="E6" s="7"/>
+      <c r="F6">
+        <f t="shared" ref="F6:F35" si="0">B6/D6</f>
+        <v>6.2373184762851057</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>12000000</v>
+      </c>
+      <c r="B7">
+        <v>5.4632949999999996</v>
+      </c>
+      <c r="C7" s="7"/>
+      <c r="D7">
+        <v>0.84793499999999999</v>
+      </c>
+      <c r="E7" s="7"/>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>6.4430587250201956</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>13000000</v>
+      </c>
+      <c r="B8">
+        <v>6.0686730000000004</v>
+      </c>
+      <c r="C8" s="7"/>
+      <c r="D8">
+        <v>0.93635000000000002</v>
+      </c>
+      <c r="E8" s="7"/>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>6.4812014738078716</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>14000000</v>
+      </c>
+      <c r="B9">
+        <v>6.7864820000000003</v>
+      </c>
+      <c r="C9" s="7"/>
+      <c r="D9">
+        <v>1.0725750000000001</v>
+      </c>
+      <c r="E9" s="7"/>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>6.3272796774118358</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
         <v>15000000</v>
       </c>
-      <c r="B6">
-        <v>7.627834</v>
-      </c>
-      <c r="C6">
-        <f>8.309336+B6</f>
-        <v>15.93717</v>
-      </c>
-      <c r="D6">
-        <v>1.166452</v>
-      </c>
-      <c r="E6">
-        <v>7.507098</v>
-      </c>
-      <c r="F6">
-        <f t="shared" ref="F6:F13" si="0">B6/D6</f>
-        <v>6.5393466683584061</v>
-      </c>
-      <c r="G6" s="5">
-        <v>2.2352059999999998</v>
-      </c>
-      <c r="H6" s="5">
-        <v>9.9260079999999995</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="2">
+      <c r="B10">
+        <v>7.5130920000000003</v>
+      </c>
+      <c r="C10" s="7"/>
+      <c r="D10">
+        <v>1.16066</v>
+      </c>
+      <c r="E10" s="7"/>
+      <c r="F10">
+        <f t="shared" si="0"/>
+        <v>6.4731204659417916</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="2">
+        <v>16000000</v>
+      </c>
+      <c r="B11">
+        <v>8.2434170000000009</v>
+      </c>
+      <c r="C11" s="7"/>
+      <c r="D11">
+        <v>1.268275</v>
+      </c>
+      <c r="E11" s="7"/>
+      <c r="F11">
+        <f t="shared" si="0"/>
+        <v>6.4997078709270468</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="2">
+        <v>17000000</v>
+      </c>
+      <c r="B12">
+        <v>9.0389809999999997</v>
+      </c>
+      <c r="C12" s="7"/>
+      <c r="D12">
+        <v>1.3796630000000001</v>
+      </c>
+      <c r="E12" s="7"/>
+      <c r="F12">
+        <f t="shared" si="0"/>
+        <v>6.5515861482115554</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="2">
+        <v>18000000</v>
+      </c>
+      <c r="B13">
+        <v>11.076497</v>
+      </c>
+      <c r="C13" s="7"/>
+      <c r="D13">
+        <v>1.566074</v>
+      </c>
+      <c r="E13" s="7"/>
+      <c r="F13">
+        <f t="shared" si="0"/>
+        <v>7.0727800857430747</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="2">
+        <v>19000000</v>
+      </c>
+      <c r="B14">
+        <v>11.668153999999999</v>
+      </c>
+      <c r="C14" s="7"/>
+      <c r="D14">
+        <v>1.6360399999999999</v>
+      </c>
+      <c r="E14" s="7"/>
+      <c r="F14">
+        <f t="shared" si="0"/>
+        <v>7.1319490965991053</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="2">
         <v>20000000</v>
       </c>
-      <c r="B7">
-        <v>11.705761000000001</v>
-      </c>
-      <c r="C7">
-        <f>10.886813+B7</f>
-        <v>22.592573999999999</v>
-      </c>
-      <c r="D7">
-        <v>1.764826</v>
-      </c>
-      <c r="E7">
-        <v>10.757872000000001</v>
-      </c>
-      <c r="F7">
-        <f t="shared" si="0"/>
-        <v>6.6328130931887905</v>
-      </c>
-      <c r="G7" s="5">
-        <v>2.9332560000000001</v>
-      </c>
-      <c r="H7" s="5">
-        <v>13.217007000000001</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="2">
+      <c r="B15">
+        <v>12.374013</v>
+      </c>
+      <c r="C15" s="7"/>
+      <c r="D15">
+        <v>1.75071</v>
+      </c>
+      <c r="E15" s="7"/>
+      <c r="F15">
+        <f t="shared" si="0"/>
+        <v>7.0679969840807439</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="2">
+        <v>21000000</v>
+      </c>
+      <c r="B16">
+        <v>13.410712999999999</v>
+      </c>
+      <c r="C16" s="7"/>
+      <c r="D16">
+        <v>1.9254990000000001</v>
+      </c>
+      <c r="E16" s="7"/>
+      <c r="F16">
+        <f t="shared" si="0"/>
+        <v>6.9647987352888778</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" s="2">
+        <v>22000000</v>
+      </c>
+      <c r="B17">
+        <v>13.503204</v>
+      </c>
+      <c r="C17" s="7"/>
+      <c r="D17">
+        <v>2.0128330000000001</v>
+      </c>
+      <c r="E17" s="7"/>
+      <c r="F17">
+        <f t="shared" si="0"/>
+        <v>6.708556546916709</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" s="2">
+        <v>23000000</v>
+      </c>
+      <c r="B18">
+        <v>15.334875</v>
+      </c>
+      <c r="C18" s="7"/>
+      <c r="D18">
+        <v>2.1030869999999999</v>
+      </c>
+      <c r="E18" s="7"/>
+      <c r="F18">
+        <f t="shared" si="0"/>
+        <v>7.2916027724958603</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="2">
+        <v>24000000</v>
+      </c>
+      <c r="B19">
+        <v>15.795399</v>
+      </c>
+      <c r="C19" s="7"/>
+      <c r="D19">
+        <v>2.2671899999999998</v>
+      </c>
+      <c r="E19" s="7"/>
+      <c r="F19">
+        <f t="shared" si="0"/>
+        <v>6.9669498365818487</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" s="2">
         <v>25000000</v>
       </c>
-      <c r="B8">
-        <v>15.923990999999999</v>
-      </c>
-      <c r="C8">
-        <f>12.898962+B8</f>
-        <v>28.822952999999998</v>
-      </c>
-      <c r="D8">
-        <v>2.3757739999999998</v>
-      </c>
-      <c r="E8">
-        <v>13.035807999999999</v>
-      </c>
-      <c r="F8">
-        <f t="shared" si="0"/>
-        <v>6.7026539561422931</v>
-      </c>
-      <c r="G8" s="5">
-        <v>3.5631789999999999</v>
-      </c>
-      <c r="H8" s="5">
-        <v>16.510265</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="2">
+      <c r="B20">
+        <v>17.032720999999999</v>
+      </c>
+      <c r="C20" s="7"/>
+      <c r="D20">
+        <v>2.413516</v>
+      </c>
+      <c r="E20" s="7"/>
+      <c r="F20">
+        <f t="shared" si="0"/>
+        <v>7.0572231549324718</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" s="2">
+        <v>26000000</v>
+      </c>
+      <c r="B21">
+        <v>18.229096999999999</v>
+      </c>
+      <c r="C21" s="7"/>
+      <c r="D21">
+        <v>2.524848</v>
+      </c>
+      <c r="E21" s="7"/>
+      <c r="F21">
+        <f t="shared" si="0"/>
+        <v>7.2198789788533801</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" s="2">
+        <v>27000000</v>
+      </c>
+      <c r="B22">
+        <v>19.070878</v>
+      </c>
+      <c r="C22" s="7"/>
+      <c r="D22">
+        <v>2.716825</v>
+      </c>
+      <c r="E22" s="7"/>
+      <c r="F22">
+        <f t="shared" si="0"/>
+        <v>7.0195459773816866</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" s="2">
+        <v>28000000</v>
+      </c>
+      <c r="B23">
+        <v>20.289345000000001</v>
+      </c>
+      <c r="C23" s="7"/>
+      <c r="D23">
+        <v>2.8388429999999998</v>
+      </c>
+      <c r="E23" s="7"/>
+      <c r="F23">
+        <f t="shared" si="0"/>
+        <v>7.1470472301567938</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="2">
+        <v>29000000</v>
+      </c>
+      <c r="B24">
+        <v>20.676687000000001</v>
+      </c>
+      <c r="C24" s="7"/>
+      <c r="D24">
+        <v>2.9750390000000002</v>
+      </c>
+      <c r="E24" s="7"/>
+      <c r="F24">
+        <f t="shared" si="0"/>
+        <v>6.9500557807813612</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="2">
         <v>30000000</v>
       </c>
-      <c r="B9">
-        <v>20.415963000000001</v>
-      </c>
-      <c r="C9">
-        <f>15.466003+B9</f>
-        <v>35.881966000000006</v>
-      </c>
-      <c r="D9">
-        <v>3.0230920000000001</v>
-      </c>
-      <c r="E9">
-        <v>15.552023999999999</v>
-      </c>
-      <c r="F9">
-        <f t="shared" si="0"/>
-        <v>6.7533383039616393</v>
-      </c>
-      <c r="G9" s="5">
-        <v>4.2926489999999999</v>
-      </c>
-      <c r="H9" s="5">
-        <v>19.987759</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="2">
+      <c r="B25">
+        <v>21.899799999999999</v>
+      </c>
+      <c r="C25" s="7"/>
+      <c r="D25">
+        <v>3.0683389999999999</v>
+      </c>
+      <c r="E25" s="7"/>
+      <c r="F25">
+        <f t="shared" si="0"/>
+        <v>7.1373469489518593</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="2">
+        <v>31000000</v>
+      </c>
+      <c r="B26">
+        <v>22.377856999999999</v>
+      </c>
+      <c r="C26" s="7"/>
+      <c r="D26">
+        <v>3.2272479999999999</v>
+      </c>
+      <c r="E26" s="7"/>
+      <c r="F26">
+        <f t="shared" si="0"/>
+        <v>6.9340369875510026</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="2">
+        <v>32000000</v>
+      </c>
+      <c r="B27">
+        <v>24.132621</v>
+      </c>
+      <c r="C27" s="7"/>
+      <c r="D27">
+        <v>3.381545</v>
+      </c>
+      <c r="E27" s="7"/>
+      <c r="F27">
+        <f t="shared" si="0"/>
+        <v>7.1365665694231479</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="2">
+        <v>33000000</v>
+      </c>
+      <c r="B28">
+        <v>24.831582999999998</v>
+      </c>
+      <c r="C28" s="7"/>
+      <c r="D28">
+        <v>3.4923199999999999</v>
+      </c>
+      <c r="E28" s="7"/>
+      <c r="F28">
+        <f t="shared" si="0"/>
+        <v>7.1103401177440784</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" s="2">
+        <v>34000000</v>
+      </c>
+      <c r="B29">
+        <v>26.061553</v>
+      </c>
+      <c r="C29" s="7"/>
+      <c r="D29">
+        <v>3.6668919999999998</v>
+      </c>
+      <c r="E29" s="7"/>
+      <c r="F29">
+        <f t="shared" si="0"/>
+        <v>7.1072594993253144</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" s="2">
         <v>35000000</v>
       </c>
-      <c r="B10">
-        <v>25.999472999999998</v>
-      </c>
-      <c r="C10">
-        <f>20.972771+B10</f>
-        <v>46.972244000000003</v>
-      </c>
-      <c r="D10">
-        <v>3.8592249999999999</v>
-      </c>
-      <c r="E10">
-        <v>18.931266000000001</v>
-      </c>
-      <c r="F10">
-        <f t="shared" si="0"/>
-        <v>6.7369673963036618</v>
-      </c>
-      <c r="G10" s="5">
-        <v>5.0395729999999999</v>
-      </c>
-      <c r="H10" s="5">
-        <v>23.276264000000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" s="2">
+      <c r="B30">
+        <v>27.901105000000001</v>
+      </c>
+      <c r="C30" s="7"/>
+      <c r="D30">
+        <v>3.7689819999999998</v>
+      </c>
+      <c r="E30" s="7"/>
+      <c r="F30">
+        <f t="shared" si="0"/>
+        <v>7.4028225658811859</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" s="2">
+        <v>36000000</v>
+      </c>
+      <c r="B31">
+        <v>28.604783999999999</v>
+      </c>
+      <c r="C31" s="7"/>
+      <c r="D31">
+        <v>4.518008</v>
+      </c>
+      <c r="E31" s="7"/>
+      <c r="F31">
+        <f t="shared" si="0"/>
+        <v>6.3312822819260166</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" s="2">
+        <v>37000000</v>
+      </c>
+      <c r="B32">
+        <v>29.860191</v>
+      </c>
+      <c r="C32" s="7"/>
+      <c r="D32">
+        <v>5.2665649999999999</v>
+      </c>
+      <c r="E32" s="7"/>
+      <c r="F32">
+        <f t="shared" si="0"/>
+        <v>5.6697659670012621</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="2">
+        <v>38000000</v>
+      </c>
+      <c r="B33">
+        <v>30.595779</v>
+      </c>
+      <c r="C33" s="7"/>
+      <c r="D33">
+        <v>4.8746859999999996</v>
+      </c>
+      <c r="E33" s="7"/>
+      <c r="F33">
+        <f t="shared" si="0"/>
+        <v>6.276461499263748</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" s="2">
+        <v>39000000</v>
+      </c>
+      <c r="B34">
+        <v>30.810445000000001</v>
+      </c>
+      <c r="C34" s="7"/>
+      <c r="D34">
+        <v>4.905627</v>
+      </c>
+      <c r="E34" s="7"/>
+      <c r="F34">
+        <f t="shared" si="0"/>
+        <v>6.2806334440021638</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" s="2">
         <v>40000000</v>
       </c>
-      <c r="B11">
-        <v>32.189481999999998</v>
-      </c>
-      <c r="C11">
-        <f>25.823072+B11</f>
-        <v>58.012553999999994</v>
-      </c>
-      <c r="D11">
-        <v>4.5912519999999999</v>
-      </c>
-      <c r="E11">
-        <v>25.360261000000001</v>
-      </c>
-      <c r="F11">
-        <f t="shared" si="0"/>
-        <v>7.0110466600395709</v>
-      </c>
-      <c r="G11" s="5">
-        <v>5.6888629999999996</v>
-      </c>
-      <c r="H11" s="5">
-        <v>25.529710000000001</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" s="2">
-        <v>45000000</v>
-      </c>
-      <c r="B12">
-        <v>37.943916999999999</v>
-      </c>
-      <c r="C12">
-        <f>29.341272+B12</f>
-        <v>67.285189000000003</v>
-      </c>
-      <c r="D12">
-        <v>5.3966729999999998</v>
-      </c>
-      <c r="E12">
-        <v>28.095462000000001</v>
-      </c>
-      <c r="F12">
-        <f t="shared" si="0"/>
-        <v>7.0309831631451454</v>
-      </c>
-      <c r="G12" s="5">
-        <v>6.5045169999999999</v>
-      </c>
-      <c r="H12" s="5">
-        <v>29.8569</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A13" s="2">
-        <v>50000000</v>
-      </c>
-      <c r="B13">
-        <v>46.904995</v>
-      </c>
-      <c r="C13">
-        <f>31.02748+B13</f>
-        <v>77.932474999999997</v>
-      </c>
-      <c r="D13">
-        <v>6.2771439999999998</v>
-      </c>
-      <c r="E13">
-        <v>31.271104000000001</v>
-      </c>
-      <c r="F13">
-        <f t="shared" si="0"/>
-        <v>7.4723465002555303</v>
-      </c>
-      <c r="G13" s="5">
-        <v>7.2976419999999997</v>
-      </c>
-      <c r="H13" s="5">
-        <v>35.428055000000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="32" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
+      <c r="B35">
+        <v>32.276363000000003</v>
+      </c>
+      <c r="C35" s="7"/>
+      <c r="D35">
+        <v>5.2940889999999996</v>
+      </c>
+      <c r="E35" s="7"/>
+      <c r="F35">
+        <f t="shared" si="0"/>
+        <v>6.0966793342537322</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B16" s="7" t="s">
+      <c r="B37" s="1"/>
+      <c r="C37" s="1"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B38" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7" t="s">
+      <c r="C38" s="8"/>
+      <c r="D38" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H16" s="6"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A17" s="3" t="s">
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B39" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C39" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D39" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E39" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="F39" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G17" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A18" s="2">
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" s="2">
         <v>10000000</v>
       </c>
-      <c r="B18">
-        <v>3.778915</v>
-      </c>
-      <c r="C18">
-        <v>8.6425140000000003</v>
-      </c>
-      <c r="D18">
-        <v>0.188636</v>
-      </c>
-      <c r="E18">
-        <v>4.9392230000000001</v>
-      </c>
-      <c r="F18">
-        <f>B18/D18</f>
-        <v>20.032841027163425</v>
-      </c>
-      <c r="G18" s="5">
-        <v>1.384317</v>
-      </c>
-      <c r="H18" s="5">
-        <v>6.1650879999999999</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A19" s="2">
+      <c r="C40" s="7"/>
+      <c r="E40" s="7"/>
+      <c r="F40" t="e">
+        <f>B40/D40</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" s="2">
+        <v>11000000</v>
+      </c>
+      <c r="F41" t="e">
+        <f t="shared" ref="F41:F70" si="1">B41/D41</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" s="2">
+        <v>12000000</v>
+      </c>
+      <c r="F42" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" s="2">
+        <v>13000000</v>
+      </c>
+      <c r="F43" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A44" s="2">
+        <v>14000000</v>
+      </c>
+      <c r="F44" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A45" s="2">
         <v>15000000</v>
       </c>
-      <c r="B19">
-        <v>6.2206219999999997</v>
-      </c>
-      <c r="C19">
-        <v>13.401472999999999</v>
-      </c>
-      <c r="D19">
-        <v>0.30043999999999998</v>
-      </c>
-      <c r="E19">
-        <v>8.0359610000000004</v>
-      </c>
-      <c r="F19">
-        <f t="shared" ref="F19:F26" si="1">B19/D19</f>
-        <v>20.705039275728932</v>
-      </c>
-      <c r="G19" s="5">
-        <v>2.5880679999999998</v>
-      </c>
-      <c r="H19" s="5">
-        <v>10.625273</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A20" s="2">
+      <c r="F45" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" s="2">
+        <v>16000000</v>
+      </c>
+      <c r="F46" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A47" s="2">
+        <v>17000000</v>
+      </c>
+      <c r="F47" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A48" s="2">
+        <v>18000000</v>
+      </c>
+      <c r="F48" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A49" s="2">
+        <v>19000000</v>
+      </c>
+      <c r="F49" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A50" s="2">
         <v>20000000</v>
       </c>
-      <c r="B20">
-        <v>10.102762</v>
-      </c>
-      <c r="C20">
-        <v>19.441248000000002</v>
-      </c>
-      <c r="D20">
-        <v>0.446938</v>
-      </c>
-      <c r="E20">
-        <v>10.283652</v>
-      </c>
-      <c r="F20">
-        <f t="shared" si="1"/>
-        <v>22.604392555566992</v>
-      </c>
-      <c r="G20" s="5">
-        <v>2.7769949999999999</v>
-      </c>
-      <c r="H20" s="5">
-        <v>12.613759999999999</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A21" s="2">
+      <c r="F50" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A51" s="2">
+        <v>21000000</v>
+      </c>
+      <c r="F51" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A52" s="2">
+        <v>22000000</v>
+      </c>
+      <c r="F52" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A53" s="2">
+        <v>23000000</v>
+      </c>
+      <c r="F53" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A54" s="2">
+        <v>24000000</v>
+      </c>
+      <c r="F54" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A55" s="2">
         <v>25000000</v>
       </c>
-      <c r="B21">
-        <v>13.203678</v>
-      </c>
-      <c r="C21">
-        <v>25.747924000000001</v>
-      </c>
-      <c r="D21">
-        <v>0.60850400000000004</v>
-      </c>
-      <c r="E21">
-        <v>11.7872</v>
-      </c>
-      <c r="F21">
-        <f t="shared" si="1"/>
-        <v>21.698588669918355</v>
-      </c>
-      <c r="G21" s="5">
-        <v>3.9838559999999998</v>
-      </c>
-      <c r="H21" s="5">
-        <v>16.541592000000001</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A22" s="2">
+      <c r="F55" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A56" s="2">
+        <v>26000000</v>
+      </c>
+      <c r="F56" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A57" s="2">
+        <v>27000000</v>
+      </c>
+      <c r="F57" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A58" s="2">
+        <v>28000000</v>
+      </c>
+      <c r="F58" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A59" s="2">
+        <v>29000000</v>
+      </c>
+      <c r="F59" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A60" s="2">
         <v>30000000</v>
       </c>
-      <c r="B22">
-        <v>17.911546000000001</v>
-      </c>
-      <c r="C22">
-        <v>30.626833000000001</v>
-      </c>
-      <c r="D22">
-        <v>0.78666400000000003</v>
-      </c>
-      <c r="E22">
-        <v>16.037421999999999</v>
-      </c>
-      <c r="F22">
-        <f t="shared" si="1"/>
-        <v>22.768991589801999</v>
-      </c>
-      <c r="G22" s="5">
-        <v>5.5545479999999996</v>
-      </c>
-      <c r="H22" s="5">
-        <v>19.275448000000001</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A23" s="2">
+      <c r="F60" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A61" s="2">
+        <v>31000000</v>
+      </c>
+      <c r="F61" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A62" s="2">
+        <v>32000000</v>
+      </c>
+      <c r="F62" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A63" s="2">
+        <v>33000000</v>
+      </c>
+      <c r="F63" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A64" s="2">
+        <v>34000000</v>
+      </c>
+      <c r="F64" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A65" s="2">
         <v>35000000</v>
       </c>
-      <c r="B23">
-        <v>19.685684999999999</v>
-      </c>
-      <c r="C23">
-        <v>35.967072999999999</v>
-      </c>
-      <c r="D23">
-        <v>0.97917200000000004</v>
-      </c>
-      <c r="E23">
-        <v>16.859352000000001</v>
-      </c>
-      <c r="F23">
-        <f t="shared" si="1"/>
-        <v>20.10441985677695</v>
-      </c>
-      <c r="G23" s="5">
-        <v>6.1012940000000002</v>
-      </c>
-      <c r="H23" s="5">
-        <v>22.961316</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A24" s="2">
+      <c r="F65" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A66" s="2">
+        <v>36000000</v>
+      </c>
+      <c r="F66" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A67" s="2">
+        <v>37000000</v>
+      </c>
+      <c r="F67" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A68" s="2">
+        <v>38000000</v>
+      </c>
+      <c r="F68" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A69" s="2">
+        <v>39000000</v>
+      </c>
+      <c r="F69" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A70" s="2">
         <v>40000000</v>
       </c>
-      <c r="B24">
-        <v>26.964960999999999</v>
-      </c>
-      <c r="C24">
-        <v>47.716700000000003</v>
-      </c>
-      <c r="D24">
-        <v>1.135345</v>
-      </c>
-      <c r="E24">
-        <v>22.491413999999999</v>
-      </c>
-      <c r="F24">
-        <f t="shared" si="1"/>
-        <v>23.750455588389432</v>
-      </c>
-      <c r="G24" s="5">
-        <v>6.5744150000000001</v>
-      </c>
-      <c r="H24" s="5">
-        <v>25.531298</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A25" s="2">
-        <v>45000000</v>
-      </c>
-      <c r="B25">
-        <v>31.982582000000001</v>
-      </c>
-      <c r="C25">
-        <v>55.762712000000001</v>
-      </c>
-      <c r="D25">
-        <v>1.3597349999999999</v>
-      </c>
-      <c r="E25">
-        <v>24.880361000000001</v>
-      </c>
-      <c r="F25">
-        <f t="shared" si="1"/>
-        <v>23.52118758434548</v>
-      </c>
-      <c r="G25" s="5">
-        <v>7.7472500000000002</v>
-      </c>
-      <c r="H25" s="5">
-        <v>31.823687</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A26" s="2">
-        <v>50000000</v>
-      </c>
-      <c r="B26">
-        <v>33.868523000000003</v>
-      </c>
-      <c r="C26">
-        <v>57.504927000000002</v>
-      </c>
-      <c r="D26">
-        <v>1.552114</v>
-      </c>
-      <c r="E26">
-        <v>25.495045000000001</v>
-      </c>
-      <c r="F26">
-        <f t="shared" si="1"/>
-        <v>21.820899109214917</v>
-      </c>
-      <c r="G26" s="5">
-        <v>9.0593489999999992</v>
-      </c>
-      <c r="H26" s="5">
-        <v>31.419589999999999</v>
+      <c r="F70" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="G16:H16"/>
+  <mergeCells count="4">
     <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B38:C38"/>
     <mergeCell ref="D3:F3"/>
-    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D38:F38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1046,15 +1347,15 @@
       <c r="B3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="6" t="s">
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="6"/>
+      <c r="G3" s="9"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -1237,15 +1538,15 @@
       <c r="B14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="6" t="s">
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G14" s="6"/>
+      <c r="G14" s="9"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">

</xml_diff>